<commit_message>
Add header, hero-media blocks, update importer
Automated migration updates generated by Experience Modernization Agent.

Changed files (6):
- blocks/header/header.css
- blocks/hero-media/hero-media.css
- tools/importer/import-home.bundle.js
- tools/importer/reports/frescopa-atelier/index.report.json
- tools/importer/reports/import-home.report.xlsx
- tools/importer/transformers/frescopa-cleanup.js
</commit_message>
<xml_diff>
--- a/tools/importer/reports/import-home.report.xlsx
+++ b/tools/importer/reports/import-home.report.xlsx
@@ -52,7 +52,7 @@
     <t>beverages</t>
   </si>
   <si>
-    <t>2026-07-15T06:31:24.065Z</t>
+    <t>2026-07-15T07:24:15.144Z</t>
   </si>
   <si>
     <t/>
@@ -73,7 +73,7 @@
     <t>blog</t>
   </si>
   <si>
-    <t>2026-07-15T06:31:34.107Z</t>
+    <t>2026-07-15T07:09:05.875Z</t>
   </si>
   <si>
     <t>https://markszulc.github.io/frescopa-atelier/blog.html</t>
@@ -91,7 +91,7 @@
     <t>cafe</t>
   </si>
   <si>
-    <t>2026-07-15T06:31:29.233Z</t>
+    <t>2026-07-15T07:09:01.080Z</t>
   </si>
   <si>
     <t>https://markszulc.github.io/frescopa-atelier/cafe.html</t>
@@ -109,7 +109,7 @@
     <t>home</t>
   </si>
   <si>
-    <t>2026-07-15T07:08:51.322Z</t>
+    <t>2026-07-15T08:53:11.807Z</t>
   </si>
   <si>
     <t>Fréscopa Atelier — Every morning, perfected.</t>

</xml_diff>